<commit_message>
Mudança nos parâmetros de custo
</commit_message>
<xml_diff>
--- a/Resultados_planta_custos_emissoes_hubs.xlsx
+++ b/Resultados_planta_custos_emissoes_hubs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epegovbr-my.sharepoint.com/personal/otto_hebeda_epe_gov_br/Documents/Documentos/Resíduos - projetos/Residuos na produção de cimento/Código/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_88B55A31088DCF73299E7AD3AB8741A67D8A8A46" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FDB0AC7-46E5-43DA-9198-EB36E7C13FA3}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_88B55A31088DCF73299E7AD3AB8741A67D8A8A46" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{967E8E64-8B2F-43A2-82AC-DF74BDC29194}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23640" yWindow="1560" windowWidth="18900" windowHeight="10965" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raio" sheetId="1" r:id="rId1"/>
@@ -533,7 +533,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -599,7 +599,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1445,6 +1445,7 @@
     <col min="17" max="17" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="27" customWidth="1"/>
     <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>